<commit_message>
Update HundredPatches multi analysis outputs
</commit_message>
<xml_diff>
--- a/Compute-Link-Attenuations/TenPatches/batch_analyze_output_multi/stats_multi.xlsx
+++ b/Compute-Link-Attenuations/TenPatches/batch_analyze_output_multi/stats_multi.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,11 @@
           <t>E_all</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>E2_all</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -502,6 +507,9 @@
       <c r="H2" t="n">
         <v>0.005115147734703691</v>
       </c>
+      <c r="I2" t="n">
+        <v>0.0006222970616919406</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -530,6 +538,9 @@
       <c r="H3" t="n">
         <v>0.005961322652001728</v>
       </c>
+      <c r="I3" t="n">
+        <v>0.001076203680393967</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -558,6 +569,9 @@
       <c r="H4" t="n">
         <v>0.001057875626004603</v>
       </c>
+      <c r="I4" t="n">
+        <v>0.001674784254147365</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -586,6 +600,9 @@
       <c r="H5" t="n">
         <v>0.003664818332437939</v>
       </c>
+      <c r="I5" t="n">
+        <v>0.0007763014199406654</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -614,6 +631,9 @@
       <c r="H6" t="n">
         <v>-0.00302430417074996</v>
       </c>
+      <c r="I6" t="n">
+        <v>0.002747724766083882</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -642,6 +662,9 @@
       <c r="H7" t="n">
         <v>0.003125549233203863</v>
       </c>
+      <c r="I7" t="n">
+        <v>0.0008693580507599857</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -670,6 +693,9 @@
       <c r="H8" t="n">
         <v>0.002051478504188021</v>
       </c>
+      <c r="I8" t="n">
+        <v>0.0005760841273232297</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -698,6 +724,9 @@
       <c r="H9" t="n">
         <v>-0.001687862501400475</v>
       </c>
+      <c r="I9" t="n">
+        <v>0.001720425713696153</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -726,6 +755,9 @@
       <c r="H10" t="n">
         <v>0.003531064188996554</v>
       </c>
+      <c r="I10" t="n">
+        <v>0.0006373250762595202</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -753,6 +785,9 @@
       </c>
       <c r="H11" t="n">
         <v>0.003706254201615038</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.000693118752020537</v>
       </c>
     </row>
   </sheetData>
@@ -47496,7 +47531,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>wet (pred &gt;= threshold)</t>
+          <t>wet (gt &gt;= threshold)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -47543,7 +47578,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>wet (pred &gt;= threshold)</t>
+          <t>wet (gt &gt;= threshold)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -47590,7 +47625,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>wet (pred &gt;= threshold)</t>
+          <t>wet (gt &gt;= threshold)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -47637,7 +47672,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>wet (pred &gt;= threshold)</t>
+          <t>wet (gt &gt;= threshold)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -47684,7 +47719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47728,6 +47763,11 @@
           <t>E_all</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>E2_all</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -47756,6 +47796,9 @@
       <c r="H2" t="n">
         <v>0.004737094557220646</v>
       </c>
+      <c r="I2" t="n">
+        <v>0.000531833297510217</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -47784,6 +47827,9 @@
       <c r="H3" t="n">
         <v>0.006027665110847955</v>
       </c>
+      <c r="I3" t="n">
+        <v>0.001095392134377851</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -47812,6 +47858,9 @@
       <c r="H4" t="n">
         <v>0.001194488329483568</v>
       </c>
+      <c r="I4" t="n">
+        <v>0.001346351402030888</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -47840,6 +47889,9 @@
       <c r="H5" t="n">
         <v>0.003783641048363989</v>
       </c>
+      <c r="I5" t="n">
+        <v>0.0008017132786392428</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -47868,6 +47920,9 @@
       <c r="H6" t="n">
         <v>-0.002914648603188149</v>
       </c>
+      <c r="I6" t="n">
+        <v>0.00188272455506917</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -47896,6 +47951,9 @@
       <c r="H7" t="n">
         <v>0.003097347417206426</v>
       </c>
+      <c r="I7" t="n">
+        <v>0.0008256550433253247</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -47924,6 +47982,9 @@
       <c r="H8" t="n">
         <v>0.002244445933802667</v>
       </c>
+      <c r="I8" t="n">
+        <v>0.0005665642979026886</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -47952,6 +48013,9 @@
       <c r="H9" t="n">
         <v>-0.001566201099833023</v>
       </c>
+      <c r="I9" t="n">
+        <v>0.001059448052006112</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -47980,6 +48044,9 @@
       <c r="H10" t="n">
         <v>0.003576921802845029</v>
       </c>
+      <c r="I10" t="n">
+        <v>0.0006630143512268025</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -48007,6 +48074,9 @@
       </c>
       <c r="H11" t="n">
         <v>0.003636988923439474</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.0006946981794490566</v>
       </c>
     </row>
   </sheetData>
@@ -48020,7 +48090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48064,6 +48134,11 @@
           <t>E_all</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>E2_all</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -48092,6 +48167,9 @@
       <c r="H2" t="n">
         <v>0.001364595220814024</v>
       </c>
+      <c r="I2" t="n">
+        <v>0.002252162526822577</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -48120,6 +48198,9 @@
       <c r="H3" t="n">
         <v>0.003365315744706829</v>
       </c>
+      <c r="I3" t="n">
+        <v>0.005134370931684691</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -48148,6 +48229,9 @@
       <c r="H4" t="n">
         <v>-0.0003464930755406259</v>
       </c>
+      <c r="I4" t="n">
+        <v>0.03714779125229746</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -48176,6 +48260,9 @@
       <c r="H5" t="n">
         <v>0.002668731219213252</v>
       </c>
+      <c r="I5" t="n">
+        <v>0.01183278426974612</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -48204,6 +48291,9 @@
       <c r="H6" t="n">
         <v>0.002372721791010654</v>
       </c>
+      <c r="I6" t="n">
+        <v>0.04597543451683309</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -48232,6 +48322,9 @@
       <c r="H7" t="n">
         <v>0.008117334010060042</v>
       </c>
+      <c r="I7" t="n">
+        <v>0.01527877507930473</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -48260,6 +48353,9 @@
       <c r="H8" t="n">
         <v>-0.004892922021564123</v>
       </c>
+      <c r="I8" t="n">
+        <v>0.02856143332693761</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -48288,6 +48384,9 @@
       <c r="H9" t="n">
         <v>-0.003203590019715465</v>
       </c>
+      <c r="I9" t="n">
+        <v>0.01694734780984011</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -48316,6 +48415,9 @@
       <c r="H10" t="n">
         <v>-0.003212918397939285</v>
       </c>
+      <c r="I10" t="n">
+        <v>0.00729838517625174</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -48343,6 +48445,9 @@
       </c>
       <c r="H11" t="n">
         <v>0.001844379130187991</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.007097127331009232</v>
       </c>
     </row>
   </sheetData>
@@ -48356,7 +48461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48400,6 +48505,11 @@
           <t>E_all</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>E2_all</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -48428,6 +48538,9 @@
       <c r="H2" t="n">
         <v>-2.860415774315879e-05</v>
       </c>
+      <c r="I2" t="n">
+        <v>5.701096970112061e-05</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -48456,6 +48569,9 @@
       <c r="H3" t="n">
         <v>-0.0005210501509056015</v>
       </c>
+      <c r="I3" t="n">
+        <v>0.0001984949020040664</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -48484,6 +48600,9 @@
       <c r="H4" t="n">
         <v>-0.0004791373814502451</v>
       </c>
+      <c r="I4" t="n">
+        <v>0.0008955136286526264</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -48512,6 +48631,9 @@
       <c r="H5" t="n">
         <v>-0.000386277440769455</v>
       </c>
+      <c r="I5" t="n">
+        <v>0.0003134358134263692</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -48540,6 +48662,9 @@
       <c r="H6" t="n">
         <v>-0.0005744450091487974</v>
       </c>
+      <c r="I6" t="n">
+        <v>0.002515720012241273</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -48568,6 +48693,9 @@
       <c r="H7" t="n">
         <v>-0.0008784611915105734</v>
       </c>
+      <c r="I7" t="n">
+        <v>0.0006735311823801542</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -48596,6 +48724,9 @@
       <c r="H8" t="n">
         <v>0.0006713293038393661</v>
       </c>
+      <c r="I8" t="n">
+        <v>0.001548307773713387</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -48624,6 +48755,9 @@
       <c r="H9" t="n">
         <v>-0.0003348858864490092</v>
       </c>
+      <c r="I9" t="n">
+        <v>0.0003060283956790368</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -48652,6 +48786,9 @@
       <c r="H10" t="n">
         <v>5.917579778501482e-05</v>
       </c>
+      <c r="I10" t="n">
+        <v>0.000272651428422457</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -48679,6 +48816,9 @@
       </c>
       <c r="H11" t="n">
         <v>-0.0004395068747252375</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.000236719240501938</v>
       </c>
     </row>
   </sheetData>

</xml_diff>